<commit_message>
Publications.featured 폐기 + CLAUDE.md 스키마 표를 실제 시트에 맞춤
featured 는 "대표 논문 강조" 용도로 스키마에 넣어뒀지만 확정 디자인에 그런
자리가 없어 끝내 어느 템플릿·필터에서도 읽히지 않았다. 37행 전부 FALSE 였다.
시트 열 삭제 + 스키마·주석에서 제거. 삭제 전 Publications 탭 전체를 백업했고,
TRUE 인 행이 0개임을 확인한 뒤에 지웠다.

같이 확인한 것: value_en/value_ko 도 1차 스캔에서 후보로 나왔으나 오탐이었다.
템플릿이 아니라 cms.js 가 cms.config / cms.configEn 을 만들 때 쓰는 재료다.
스캔 범위에서 데이터 계층을 빼놓은 탓이었고 후보에서 제외했다.

CLAUDE.md §5 표가 실제 시트와 여러 곳 어긋나 있었다(Publications 에 존재하지
않는 details·raw_citation, News 의 옛 열 이름, Conferences·Invited_Talks·Gallery
누락, 폐기된 Collaborators). 12개 탭 헤더를 전부 대조해 맞췄다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013UgoWvTJbXT49za1EABuA7
</commit_message>
<xml_diff>
--- a/eplab_website_content.xlsx
+++ b/eplab_website_content.xlsx
@@ -505,7 +505,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -529,16 +529,16 @@
         <v>TRUE</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>270</v>
       </c>
       <c r="C2" t="str">
-        <v>2026.03</v>
+        <v>2023.09</v>
       </c>
       <c r="D2" t="str">
-        <v>전기자동차 구동모터 개발동향 및 열관리 전략</v>
+        <v>전기자동차 파워트레인의 기술 동향</v>
       </c>
       <c r="E2" t="str">
-        <v>한양대학교</v>
+        <v>동국대학교 BK21 초청세미나</v>
       </c>
     </row>
     <row r="3">
@@ -546,16 +546,16 @@
         <v>TRUE</v>
       </c>
       <c r="B3" t="str">
-        <v>20</v>
+        <v>260</v>
       </c>
       <c r="C3" t="str">
-        <v>2025.09</v>
+        <v>2023.10</v>
       </c>
       <c r="D3" t="str">
-        <v>협동로봇 구동모듈의 PHM</v>
+        <v>전기자동차 파워트레인의 기술 동향</v>
       </c>
       <c r="E3" t="str">
-        <v>두산로보틱스</v>
+        <v>한국자동차연구원</v>
       </c>
     </row>
     <row r="4">
@@ -563,16 +563,16 @@
         <v>TRUE</v>
       </c>
       <c r="B4" t="str">
-        <v>30</v>
+        <v>250</v>
       </c>
       <c r="C4" t="str">
-        <v>2025.08</v>
+        <v>2023.12</v>
       </c>
       <c r="D4" t="str">
-        <v>Scaling 기반 모터 설계 효율화 및 심층전이학습 기반 설계/시험 효율화</v>
+        <v>전동화 파워트레인 연구동향</v>
       </c>
       <c r="E4" t="str">
-        <v>대구대학교</v>
+        <v>한국자동차연구원</v>
       </c>
     </row>
     <row r="5">
@@ -580,16 +580,16 @@
         <v>TRUE</v>
       </c>
       <c r="B5" t="str">
-        <v>40</v>
+        <v>240</v>
       </c>
       <c r="C5" t="str">
-        <v>2025.08</v>
+        <v>2024.02</v>
       </c>
       <c r="D5" t="str">
-        <v>전자기 액추에이터 기초 이론 및 실습</v>
+        <v>전기자동차 구동모터의 시험-해석 정합성 향상에 관한 연구</v>
       </c>
       <c r="E5" t="str">
-        <v>한국최적설계학회 하계강습회</v>
+        <v>서울대학교 기계공학부</v>
       </c>
     </row>
     <row r="6">
@@ -597,16 +597,16 @@
         <v>TRUE</v>
       </c>
       <c r="B6" t="str">
-        <v>50</v>
+        <v>230</v>
       </c>
       <c r="C6" t="str">
-        <v>2025.07</v>
+        <v>2024.03</v>
       </c>
       <c r="D6" t="str">
-        <v>구동모터 기초이론 및 비효율 전류벡터제어 기반 강제발열모드</v>
+        <v>전자기 유한요소해석 기반 철손해석</v>
       </c>
       <c r="E6" t="str">
-        <v>현대자동차 열에너지통합개발실</v>
+        <v>한국생산기술연구원</v>
       </c>
     </row>
     <row r="7">
@@ -614,16 +614,16 @@
         <v>TRUE</v>
       </c>
       <c r="B7" t="str">
-        <v>60</v>
+        <v>220</v>
       </c>
       <c r="C7" t="str">
-        <v>2025.07</v>
+        <v>2024.06</v>
       </c>
       <c r="D7" t="str">
-        <v>핵심 구동 부품 전자기-기계 성능 최신 연구동향</v>
+        <v>전기자동차 구동모터의 시험-해석 정합성 향상에 관한 연구</v>
       </c>
       <c r="E7" t="str">
-        <v>한국자동차연구원</v>
+        <v>영남대학교 기계공학부</v>
       </c>
     </row>
     <row r="8">
@@ -631,16 +631,16 @@
         <v>TRUE</v>
       </c>
       <c r="B8" t="str">
-        <v>70</v>
+        <v>210</v>
       </c>
       <c r="C8" t="str">
-        <v>2025.06</v>
+        <v>2024.07</v>
       </c>
       <c r="D8" t="str">
-        <v>2-Stage 인버터 토폴로지 적용 PE 시스템의 설계, 제어 및 응용</v>
+        <v>개방형 권선 구조 및 IPMSM의 전자기 성능해석 및 응용</v>
       </c>
       <c r="E8" t="str">
-        <v>현대모비스 전동화BU</v>
+        <v>한국생산기술연구원</v>
       </c>
     </row>
     <row r="9">
@@ -648,16 +648,16 @@
         <v>TRUE</v>
       </c>
       <c r="B9" t="str">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="C9" t="str">
-        <v>2025.05</v>
+        <v>2024.08</v>
       </c>
       <c r="D9" t="str">
-        <v>Scaling 기반 모터 설계 효율화 및 심층전이학습 기반 설계/시험 효율화</v>
+        <v>전기자동차 구동모터 연구개발 동향 및 고효율/고출력 구동시스템 신구조</v>
       </c>
       <c r="E9" t="str">
-        <v>LG전자</v>
+        <v>충남대학교 전기공학과</v>
       </c>
     </row>
     <row r="10">
@@ -665,16 +665,16 @@
         <v>TRUE</v>
       </c>
       <c r="B10" t="str">
-        <v>90</v>
+        <v>190</v>
       </c>
       <c r="C10" t="str">
-        <v>2025.05</v>
+        <v>2024.08</v>
       </c>
       <c r="D10" t="str">
-        <v>전동화 가속을 위한 AI 및 CAE 빅데이터 기반 구동모터 시험/설계 효율화 기술</v>
+        <v>고효율/고출력 구동시스템 신구조 및 시험-해석 가속화 연구</v>
       </c>
       <c r="E10" t="str">
-        <v>한국자동차연구원</v>
+        <v>LG전자 가산R&amp;D캠퍼스</v>
       </c>
     </row>
     <row r="11">
@@ -682,16 +682,16 @@
         <v>TRUE</v>
       </c>
       <c r="B11" t="str">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="C11" t="str">
-        <v>2025.05</v>
+        <v>2024.09</v>
       </c>
       <c r="D11" t="str">
-        <v>고효율 구동시스템을 위한 권선 토폴로지 &amp; PE 시스템의 Multi-physics 성능해석</v>
+        <v>고출력밀도 전기모터를 위한 적층제조 코일 연구동향</v>
       </c>
       <c r="E11" t="str">
-        <v>보그워너</v>
+        <v>한국생산기술연구원</v>
       </c>
     </row>
     <row r="12">
@@ -699,16 +699,16 @@
         <v>TRUE</v>
       </c>
       <c r="B12" t="str">
-        <v>110</v>
+        <v>170</v>
       </c>
       <c r="C12" t="str">
-        <v>2025.02</v>
+        <v>2024.10</v>
       </c>
       <c r="D12" t="str">
-        <v>친환경자동차 PE 시스템 권선절환 토폴로지 &amp; 전이학습 기반 시험/설계 효율화</v>
+        <v>전기자동차 구동모터의 글로벌 최신 연구 동향</v>
       </c>
       <c r="E12" t="str">
-        <v>현대자동차 전동화시험센터</v>
+        <v>한국생산기술연구원</v>
       </c>
     </row>
     <row r="13">
@@ -716,13 +716,13 @@
         <v>TRUE</v>
       </c>
       <c r="B13" t="str">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="C13" t="str">
-        <v>2024.12</v>
+        <v>2024.10</v>
       </c>
       <c r="D13" t="str">
-        <v>xEV 구동모터 개발기간 단축을 위한 설계 및 시험기술</v>
+        <v>친환경자동차 구동시스템 토폴로지</v>
       </c>
       <c r="E13" t="str">
         <v>한국자동차연구원</v>
@@ -733,13 +733,13 @@
         <v>TRUE</v>
       </c>
       <c r="B14" t="str">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="C14" t="str">
-        <v>2024.10</v>
+        <v>2024.12</v>
       </c>
       <c r="D14" t="str">
-        <v>친환경자동차 구동시스템 토폴로지</v>
+        <v>xEV 구동모터 개발기간 단축을 위한 설계 및 시험기술</v>
       </c>
       <c r="E14" t="str">
         <v>한국자동차연구원</v>
@@ -753,13 +753,13 @@
         <v>140</v>
       </c>
       <c r="C15" t="str">
-        <v>2024.10</v>
+        <v>2025.02</v>
       </c>
       <c r="D15" t="str">
-        <v>전기자동차 구동모터의 글로벌 최신 연구 동향</v>
+        <v>친환경자동차 PE 시스템 권선절환 토폴로지 &amp; 전이학습 기반 시험/설계 효율화</v>
       </c>
       <c r="E15" t="str">
-        <v>한국생산기술연구원</v>
+        <v>현대자동차 전동화시험센터</v>
       </c>
     </row>
     <row r="16">
@@ -767,16 +767,16 @@
         <v>TRUE</v>
       </c>
       <c r="B16" t="str">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C16" t="str">
-        <v>2024.09</v>
+        <v>2025.05</v>
       </c>
       <c r="D16" t="str">
-        <v>고출력밀도 전기모터를 위한 적층제조 코일 연구동향</v>
+        <v>고효율 구동시스템을 위한 권선 토폴로지 &amp; PE 시스템의 Multi-physics 성능해석</v>
       </c>
       <c r="E16" t="str">
-        <v>한국생산기술연구원</v>
+        <v>보그워너</v>
       </c>
     </row>
     <row r="17">
@@ -784,16 +784,16 @@
         <v>TRUE</v>
       </c>
       <c r="B17" t="str">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="C17" t="str">
-        <v>2024.08</v>
+        <v>2025.05</v>
       </c>
       <c r="D17" t="str">
-        <v>고효율/고출력 구동시스템 신구조 및 시험-해석 가속화 연구</v>
+        <v>전동화 가속을 위한 AI 및 CAE 빅데이터 기반 구동모터 시험/설계 효율화 기술</v>
       </c>
       <c r="E17" t="str">
-        <v>LG전자 가산R&amp;D캠퍼스</v>
+        <v>한국자동차연구원</v>
       </c>
     </row>
     <row r="18">
@@ -801,16 +801,16 @@
         <v>TRUE</v>
       </c>
       <c r="B18" t="str">
-        <v>170</v>
+        <v>110</v>
       </c>
       <c r="C18" t="str">
-        <v>2024.08</v>
+        <v>2025.05</v>
       </c>
       <c r="D18" t="str">
-        <v>전기자동차 구동모터 연구개발 동향 및 고효율/고출력 구동시스템 신구조</v>
+        <v>Scaling 기반 모터 설계 효율화 및 심층전이학습 기반 설계/시험 효율화</v>
       </c>
       <c r="E18" t="str">
-        <v>충남대학교 전기공학과</v>
+        <v>LG전자</v>
       </c>
     </row>
     <row r="19">
@@ -818,16 +818,16 @@
         <v>TRUE</v>
       </c>
       <c r="B19" t="str">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="C19" t="str">
-        <v>2024.07</v>
+        <v>2025.06</v>
       </c>
       <c r="D19" t="str">
-        <v>개방형 권선 구조 및 IPMSM의 전자기 성능해석 및 응용</v>
+        <v>2-Stage 인버터 토폴로지 적용 PE 시스템의 설계, 제어 및 응용</v>
       </c>
       <c r="E19" t="str">
-        <v>한국생산기술연구원</v>
+        <v>현대모비스 전동화BU</v>
       </c>
     </row>
     <row r="20">
@@ -835,16 +835,16 @@
         <v>TRUE</v>
       </c>
       <c r="B20" t="str">
-        <v>190</v>
+        <v>90</v>
       </c>
       <c r="C20" t="str">
-        <v>2024.06</v>
+        <v>2025.07</v>
       </c>
       <c r="D20" t="str">
-        <v>전기자동차 구동모터의 시험-해석 정합성 향상에 관한 연구</v>
+        <v>핵심 구동 부품 전자기-기계 성능 최신 연구동향</v>
       </c>
       <c r="E20" t="str">
-        <v>영남대학교 기계공학부</v>
+        <v>한국자동차연구원</v>
       </c>
     </row>
     <row r="21">
@@ -852,16 +852,16 @@
         <v>TRUE</v>
       </c>
       <c r="B21" t="str">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C21" t="str">
-        <v>2024.03</v>
+        <v>2025.07</v>
       </c>
       <c r="D21" t="str">
-        <v>전자기 유한요소해석 기반 철손해석</v>
+        <v>구동모터 기초이론 및 비효율 전류벡터제어 기반 강제발열모드</v>
       </c>
       <c r="E21" t="str">
-        <v>한국생산기술연구원</v>
+        <v>현대자동차 열에너지통합개발실</v>
       </c>
     </row>
     <row r="22">
@@ -869,16 +869,16 @@
         <v>TRUE</v>
       </c>
       <c r="B22" t="str">
-        <v>210</v>
+        <v>70</v>
       </c>
       <c r="C22" t="str">
-        <v>2024.02</v>
+        <v>2025.08</v>
       </c>
       <c r="D22" t="str">
-        <v>전기자동차 구동모터의 시험-해석 정합성 향상에 관한 연구</v>
+        <v>전자기 액추에이터 기초 이론 및 실습</v>
       </c>
       <c r="E22" t="str">
-        <v>서울대학교 기계공학부</v>
+        <v>한국최적설계학회 하계강습회</v>
       </c>
     </row>
     <row r="23">
@@ -886,16 +886,16 @@
         <v>TRUE</v>
       </c>
       <c r="B23" t="str">
-        <v>220</v>
+        <v>60</v>
       </c>
       <c r="C23" t="str">
-        <v>2023.12</v>
+        <v>2025.08</v>
       </c>
       <c r="D23" t="str">
-        <v>전동화 파워트레인 연구동향</v>
+        <v>Scaling 기반 모터 설계 효율화 및 심층전이학습 기반 설계/시험 효율화</v>
       </c>
       <c r="E23" t="str">
-        <v>한국자동차연구원</v>
+        <v>대구대학교</v>
       </c>
     </row>
     <row r="24">
@@ -903,16 +903,16 @@
         <v>TRUE</v>
       </c>
       <c r="B24" t="str">
-        <v>230</v>
+        <v>50</v>
       </c>
       <c r="C24" t="str">
-        <v>2023.10</v>
+        <v>2025.09</v>
       </c>
       <c r="D24" t="str">
-        <v>전기자동차 파워트레인의 기술 동향</v>
+        <v>협동로봇 구동모듈의 PHM</v>
       </c>
       <c r="E24" t="str">
-        <v>한국자동차연구원</v>
+        <v>두산로보틱스</v>
       </c>
     </row>
     <row r="25">
@@ -920,21 +920,72 @@
         <v>TRUE</v>
       </c>
       <c r="B25" t="str">
-        <v>240</v>
+        <v>40</v>
       </c>
       <c r="C25" t="str">
-        <v>2023.09</v>
+        <v>2026.03</v>
       </c>
       <c r="D25" t="str">
-        <v>전기자동차 파워트레인의 기술 동향</v>
+        <v>전기자동차 구동모터 개발동향 및 열관리 전략</v>
       </c>
       <c r="E25" t="str">
-        <v>동국대학교 BK21 초청세미나</v>
+        <v>한양대학교</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B26" t="str">
+        <v>30</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2026.04</v>
+      </c>
+      <c r="D26" t="str">
+        <v>전기자동차 구동모터 개발동향 및 열관리 전략</v>
+      </c>
+      <c r="E26" t="str">
+        <v>GIST</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B27" t="str">
+        <v>20</v>
+      </c>
+      <c r="C27" t="str">
+        <v>2026.07</v>
+      </c>
+      <c r="D27" t="str">
+        <v>전동화 가속을 위한 AI 및 CAE 빅데이터 기반구동모터 시험/설계 효율화 기술</v>
+      </c>
+      <c r="E27" t="str">
+        <v>한국자동차연구원</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B28" t="str">
+        <v>10</v>
+      </c>
+      <c r="C28" t="str">
+        <v>2026.08</v>
+      </c>
+      <c r="D28" t="str">
+        <v>모터 응용 분야별 열관리 기법_x000d_</v>
+      </c>
+      <c r="E28" t="str">
+        <v>PHM 리더양성을 위한 전문기술 강좌</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2189,7 +2240,7 @@
         <v>stat_researchers</v>
       </c>
       <c r="B12" t="str">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -2217,7 +2268,7 @@
         <v>stat_projects</v>
       </c>
       <c r="B14" t="str">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -3436,7 +3487,7 @@
         <v>240</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>2023 – present</v>
       </c>
       <c r="E25" t="str">
         <v>Reviewer: TIE, TMECH, TTE, TMAG, TEC, IEEE ACCESS, JEET, JOM</v>
@@ -3641,7 +3692,7 @@
         <v>TRUE</v>
       </c>
       <c r="B2" t="str">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="C2" t="str">
         <v>Completed</v>
@@ -3667,7 +3718,7 @@
         <v>TRUE</v>
       </c>
       <c r="B3" t="str">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="C3" t="str">
         <v>Completed</v>
@@ -3693,7 +3744,7 @@
         <v>TRUE</v>
       </c>
       <c r="B4" t="str">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C4" t="str">
         <v>Completed</v>
@@ -3719,7 +3770,7 @@
         <v>TRUE</v>
       </c>
       <c r="B5" t="str">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="C5" t="str">
         <v>Completed</v>
@@ -3745,7 +3796,7 @@
         <v>TRUE</v>
       </c>
       <c r="B6" t="str">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="C6" t="str">
         <v>Completed</v>
@@ -3771,7 +3822,7 @@
         <v>TRUE</v>
       </c>
       <c r="B7" t="str">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="C7" t="str">
         <v>Completed</v>
@@ -3797,7 +3848,7 @@
         <v>TRUE</v>
       </c>
       <c r="B8" t="str">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C8" t="str">
         <v>Completed</v>
@@ -3823,7 +3874,7 @@
         <v>TRUE</v>
       </c>
       <c r="B9" t="str">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="C9" t="str">
         <v>Completed</v>
@@ -3849,7 +3900,7 @@
         <v>TRUE</v>
       </c>
       <c r="B10" t="str">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="C10" t="str">
         <v>Completed</v>
@@ -3875,7 +3926,7 @@
         <v>TRUE</v>
       </c>
       <c r="B11" t="str">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="C11" t="str">
         <v>Completed</v>
@@ -3901,7 +3952,7 @@
         <v>TRUE</v>
       </c>
       <c r="B12" t="str">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="C12" t="str">
         <v>Completed</v>
@@ -3927,7 +3978,7 @@
         <v>TRUE</v>
       </c>
       <c r="B13" t="str">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C13" t="str">
         <v>Completed</v>
@@ -3953,7 +4004,7 @@
         <v>TRUE</v>
       </c>
       <c r="B14" t="str">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="C14" t="str">
         <v>Completed</v>
@@ -3982,22 +4033,22 @@
         <v>130</v>
       </c>
       <c r="C15" t="str">
-        <v>Ongoing</v>
+        <v>Completed</v>
       </c>
       <c r="D15" t="str">
-        <v>Co-I</v>
+        <v>Advisor</v>
       </c>
       <c r="E15" t="str">
-        <v>AI-핵심소재 기반 첨단산업 지능형 로봇 글로벌인재양성</v>
+        <v>다족보행로봇의 에너지효율 향상을 위한 다중물리모델 기반 구동계 최적설계기술 연구</v>
       </c>
       <c r="F15" t="str">
-        <v>한국산업기술진흥원</v>
+        <v>한국연구재단(석사과정생연구장려금지원사업)</v>
       </c>
       <c r="G15" t="str">
-        <v>2024.03</v>
+        <v>2025.09</v>
       </c>
       <c r="H15" t="str">
-        <v>2027.02</v>
+        <v>2026.09</v>
       </c>
     </row>
     <row r="16">
@@ -4008,22 +4059,22 @@
         <v>120</v>
       </c>
       <c r="C16" t="str">
-        <v>Ongoing</v>
+        <v>Completed</v>
       </c>
       <c r="D16" t="str">
-        <v>Co-I</v>
+        <v>Advisor</v>
       </c>
       <c r="E16" t="str">
-        <v>평각동선 분포권 기술 적용 축방향자속 전동기 개발</v>
+        <v>전기차 파워트레인의 데이터 주도 고장예지를 위한 고장데이터 생성 다중물리 해석모델 연구</v>
       </c>
       <c r="F16" t="str">
-        <v>효성전기 · 한국자동차연구원 · 대구대학교</v>
+        <v>한국연구재단(석사과정생연구장려금지원사업)</v>
       </c>
       <c r="G16" t="str">
-        <v>2025.04</v>
+        <v>2025.09</v>
       </c>
       <c r="H16" t="str">
-        <v>2028.12</v>
+        <v>2026.09</v>
       </c>
     </row>
     <row r="17">
@@ -4037,19 +4088,19 @@
         <v>Ongoing</v>
       </c>
       <c r="D17" t="str">
-        <v>Advisor</v>
+        <v>Co-I</v>
       </c>
       <c r="E17" t="str">
-        <v>다족보행로봇의 에너지효율 향상을 위한 다중물리모델 기반 구동계 최적설계기술 연구</v>
+        <v>AI-핵심소재 기반 첨단산업 지능형 로봇 글로벌인재양성</v>
       </c>
       <c r="F17" t="str">
-        <v>한국연구재단(석사과정생연구장려금지원사업)</v>
+        <v>한국산업기술진흥원</v>
       </c>
       <c r="G17" t="str">
-        <v>2025.09</v>
+        <v>2024.03</v>
       </c>
       <c r="H17" t="str">
-        <v>2026.09</v>
+        <v>2027.02</v>
       </c>
     </row>
     <row r="18">
@@ -4063,19 +4114,19 @@
         <v>Ongoing</v>
       </c>
       <c r="D18" t="str">
-        <v>Advisor</v>
+        <v>Co-I</v>
       </c>
       <c r="E18" t="str">
-        <v>전기차 파워트레인의 데이터 주도 고장예지를 위한 고장데이터 생성 다중물리 해석모델 연구</v>
+        <v>평각동선 분포권 기술 적용 축방향자속 전동기 개발</v>
       </c>
       <c r="F18" t="str">
-        <v>한국연구재단(석사과정생연구장려금지원사업)</v>
+        <v>한국산업기획평가원</v>
       </c>
       <c r="G18" t="str">
-        <v>2025.09</v>
+        <v>2025.04</v>
       </c>
       <c r="H18" t="str">
-        <v>2026.09</v>
+        <v>2028.12</v>
       </c>
     </row>
     <row r="19">
@@ -4274,7 +4325,7 @@
         <v>Advisor</v>
       </c>
       <c r="E26" t="str">
-        <v>Super-resolution</v>
+        <v>AI 기반 초해상도을 활용한 축방향 자속 모터의 다중 메쉬 해상도 기반 전자계 해석 가속화 연구</v>
       </c>
       <c r="F26" t="str">
         <v>한국연구재단(석사과정생연구장려금지원사업)</v>
@@ -4321,7 +4372,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:H39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4348,37 +4399,31 @@
       <c r="H1" t="str">
         <v>doi</v>
       </c>
-      <c r="I1" t="str">
-        <v>featured</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>TRUE</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>370</v>
       </c>
       <c r="C2" t="str">
-        <v>2026</v>
+        <v>2019</v>
       </c>
       <c r="D2" t="str">
-        <v>J. H. Lee, S. H. Park, D. H. Park, J. H. Jeong, and M. S. Lim*</v>
+        <v>S. H. Park, J. C. Park, J. W. Chin, H. J. Park, S. O. Kwon, S. I. Kim, and M. S. Lim*</v>
       </c>
       <c r="E2" t="str">
-        <v>Deep Transfer Learning-Based Demagnetization Analysis for Linear Oscillating Actuator Considering Circumferential Segmented Structure</v>
+        <v>Design of Surface-mounted Permanent Magnet Synchronous Motor using Electromagnetic and Thermal Analysis</v>
       </c>
       <c r="F2" t="str">
-        <v>IEEE Transactions on Industry Applications, vol. 62, no. 1, pp. 821–829, Jan. 2026</v>
+        <v>Journal of Magnetics, vol. 24, no. 4, pp. 606–615, Dec. 2019</v>
       </c>
       <c r="G2" t="str">
-        <v>IF 4.2 · Q1 · JCR 13.0%</v>
+        <v>IF 0.628 · Q4</v>
       </c>
       <c r="H2" t="str">
-        <v>https://doi.org/10.1109/TIA.2025.3585098</v>
-      </c>
-      <c r="I2" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.4283/JMAG.2019.24.4.606</v>
       </c>
     </row>
     <row r="3">
@@ -4386,28 +4431,25 @@
         <v>TRUE</v>
       </c>
       <c r="B3" t="str">
-        <v>20</v>
+        <v>360</v>
       </c>
       <c r="C3" t="str">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="D3" t="str">
-        <v>K. S. Cha**, S. H. Park**, and Y. H. Jung*</v>
+        <v>S. H. Park, J. C. Park, S. W. Hwang, J. H. Kim, H. J. Park, and M. S. Lim*</v>
       </c>
       <c r="E3" t="str">
-        <v>Design of WFSM using Sizing Method Combining 2D Equivalent Magnetic Circuit considering Nonlinear Characteristics</v>
+        <v>Suppression of Torque Ripple Caused by Misalignment of the Gearbox by Using Harmonic Current Injection Method</v>
       </c>
       <c r="F3" t="str">
-        <v>IEEE Transactions on Magnetics, Early Access, 2025</v>
+        <v>IEEE/ASME Transactions on Mechatronics, vol. 25, no. 4, pp. 1990–1999, Aug. 2020</v>
       </c>
       <c r="G3" t="str">
-        <v>IF 2.1 · Q3 · JCR 54.5%</v>
+        <v>IF 4.943 · Q1 · JCR 5.0%</v>
       </c>
       <c r="H3" t="str">
-        <v>https://doi.org/10.1109/TMAG.2025.3624623</v>
-      </c>
-      <c r="I3" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMECH.2020.2999379</v>
       </c>
     </row>
     <row r="4">
@@ -4415,28 +4457,25 @@
         <v>TRUE</v>
       </c>
       <c r="B4" t="str">
-        <v>30</v>
+        <v>350</v>
       </c>
       <c r="C4" t="str">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="D4" t="str">
-        <v>Y. M. Lee, D. H. Ko, S. Yoon, J. Cho, S. H. Park*, and M. R. Park*</v>
+        <v>S. H. Park, J. C. Park, H. Y. Lee, S. O. Kwon, and M. S. Lim*</v>
       </c>
       <c r="E4" t="str">
-        <v>Characteristics Estimation and Design of SPMSM using Analytic Method-based Transfer Learning</v>
+        <v>Design of High-Bandwidth Motor System Considering Electrical and Mechanical Time Constant</v>
       </c>
       <c r="F4" t="str">
-        <v>IEEE Transactions on Magnetics, Early Access, 2025</v>
+        <v>IEEE Transactions on Industry Applications, vol. 56, no. 5, pp. 4738–4747, Sep. 2020</v>
       </c>
       <c r="G4" t="str">
-        <v>IF 2.1 · Q3 · JCR 54.5%</v>
+        <v>IF 2.743 · Q1 · JCR 15.7%</v>
       </c>
       <c r="H4" t="str">
-        <v>https://doi.org/10.1109/TMAG.2025.3640767</v>
-      </c>
-      <c r="I4" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TIA.2020.2998674</v>
       </c>
     </row>
     <row r="5">
@@ -4444,28 +4483,25 @@
         <v>TRUE</v>
       </c>
       <c r="B5" t="str">
-        <v>40</v>
+        <v>340</v>
       </c>
       <c r="C5" t="str">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D5" t="str">
-        <v>S. H. Park, D. H. Ko, S. G. Lee, J. C. Park, and M. R. Park*</v>
+        <v>S. H. Park, E. C. Lee, J. C. Park, S. W. Hwang, and M. S. Lim*</v>
       </c>
       <c r="E5" t="str">
-        <v>Robust Design Optimization of SPMSM based on Manufacturing Uncertainty Analysis of Prototype</v>
+        <v>Prediction of Mechanical Loss for High-Power-Density PMSM Considering Eddy Current Loss of PMs and Conductors</v>
       </c>
       <c r="F5" t="str">
-        <v>IEEE Transactions on Magnetics, Early Access, 2025</v>
+        <v>IEEE Transactions on Magnetics, vol. 57, no. 2, Feb. 2021</v>
       </c>
       <c r="G5" t="str">
-        <v>IF 2.1 · Q3 · JCR 54.5%</v>
+        <v>IF 1.651 · Q3</v>
       </c>
       <c r="H5" t="str">
-        <v>https://doi.org/10.1109/TMAG.2025.3616812</v>
-      </c>
-      <c r="I5" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2020.3007439</v>
       </c>
     </row>
     <row r="6">
@@ -4473,28 +4509,25 @@
         <v>TRUE</v>
       </c>
       <c r="B6" t="str">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="C6" t="str">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D6" t="str">
-        <v>S. Khalid, J. W. Song, M. H. Yazdani, M. U. Elahi, S. H. Park, H. S. Kim*, Y. G. Yoon, and J. S. Lee</v>
+        <v>J. C. Park, S. H. Park, J. H. Kim, S. G. Lee, G. H. Lee, and M. S. Lim*</v>
       </c>
       <c r="E6" t="str">
-        <v>Advances in prognostics and health management of light emitting diodes: A comprehensive review</v>
+        <v>Diagnosis and Robust Design Optimization of SPMSM Considering Back EMF and Cogging Torque due to Static Eccentricity</v>
       </c>
       <c r="F6" t="str">
-        <v>Journal of Computational Design and Engineering, vol. 12, no. 9, pp. 184–203, Sept. 2025</v>
+        <v>Energies, vol. 14, no. 10, pp. 2900–2918, May 2021</v>
       </c>
       <c r="G6" t="str">
-        <v>IF 4.8 · Q1 · JCR 11.3%</v>
+        <v>IF 2.702 · Q3</v>
       </c>
       <c r="H6" t="str">
-        <v>https://doi.org/10.1093/jcde/qwaf090</v>
-      </c>
-      <c r="I6" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/en14102900</v>
       </c>
     </row>
     <row r="7">
@@ -4502,28 +4535,25 @@
         <v>TRUE</v>
       </c>
       <c r="B7" t="str">
-        <v>60</v>
+        <v>320</v>
       </c>
       <c r="C7" t="str">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D7" t="str">
-        <v>Y. H. Jung**, D. M. Kim**, K. S. Cha, S. H. Park*, and M. R. Park*</v>
+        <v>S. H. Park, E. C. Lee, G. J. Lee, S. O. Kwon, and M. S. Lim*</v>
       </c>
       <c r="E7" t="str">
-        <v>Vibration Reduction of Permanent Magnet Synchronous Motors by Four-Layer Winding: Mathematical Modeling and Experimental Validation</v>
+        <v>Effect of Pole and Slot Combination on the AC Joule Loss of Outer-Rotor Permanent Magnet Synchronous Motors Using a High Fill Factor Machined Coil</v>
       </c>
       <c r="F7" t="str">
-        <v>Mathematics, vol. 13, no. 9, pp. 1603–1621, May 2025</v>
+        <v>Energies, vol. 14, no. 10, pp. 3073–3083, May 2021</v>
       </c>
       <c r="G7" t="str">
-        <v>IF 2.3 · Q1 · JCR 4.2%</v>
+        <v>IF 2.702 · Q3</v>
       </c>
       <c r="H7" t="str">
-        <v>https://doi.org/10.3390/math13101603</v>
-      </c>
-      <c r="I7" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/en14113073</v>
       </c>
     </row>
     <row r="8">
@@ -4531,28 +4561,25 @@
         <v>TRUE</v>
       </c>
       <c r="B8" t="str">
-        <v>70</v>
+        <v>310</v>
       </c>
       <c r="C8" t="str">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D8" t="str">
-        <v>K. S. Cha**, Y. H. Jung**, S. H. Park*, and M. R. Park*</v>
+        <v>S. W. Hwang, J. Y. Ryu, J. W. Chin, S. H. Park, D. K. Kim, and M. S. Lim*</v>
       </c>
       <c r="E8" t="str">
-        <v>Optimal Design Considering AC Copper Loss of Traction Motor Applied HSFF Coil for Improving Electric Bus Fuel Economy</v>
+        <v>Coupled Electromagnetic-Thermal Analysis for Predicting Traction Motor Characteristics According to Electric Vehicle Driving Cycle</v>
       </c>
       <c r="F8" t="str">
-        <v>Mathematics, vol. 13, no. 9, pp. 1509–1528, May 2025</v>
+        <v>IEEE Transactions on Vehicular Technology, vol. 70, no. 5, pp. 4262–4272, May 2021</v>
       </c>
       <c r="G8" t="str">
-        <v>IF 2.3 · Q1 · JCR 4.2%</v>
+        <v>IF 5.339 · Q1 · JCR 11.1%</v>
       </c>
       <c r="H8" t="str">
-        <v>https://doi.org/10.3390/math13091509</v>
-      </c>
-      <c r="I8" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TVT.2021.3071943</v>
       </c>
     </row>
     <row r="9">
@@ -4560,28 +4587,25 @@
         <v>TRUE</v>
       </c>
       <c r="B9" t="str">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="C9" t="str">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D9" t="str">
-        <v>M. H. Sung**, S. H. Park**, K. S. Cha, J. H. Sim, and M. S. Lim*</v>
+        <v>J. W. Chin, K. S. Cha, M. R. Park, S. H. Park, E. C. Lee, and M. S. Lim*</v>
       </c>
       <c r="E9" t="str">
-        <v>Deep Transfer Learning-Based Performance Prediction Considering 3-D Flux in Outer Rotor Interior Permanent Magnet Synchronous Motors</v>
+        <v>High Efficiency PMSM With High Slot Fill Factor Coil for Heavy-Duty EV Traction Considering AC Resistance</v>
       </c>
       <c r="F9" t="str">
-        <v>Machines, vol. 13, no. 4, pp. 302–313, Apr. 2025</v>
+        <v>IEEE Transactions on Energy Conversion, vol. 36, no. 2, pp. 883–894, June 2021</v>
       </c>
       <c r="G9" t="str">
-        <v>IF 2.1 · Q2 · JCR 45.1%</v>
+        <v>IF 4.614 · Q1 · JCR 14.9%</v>
       </c>
       <c r="H9" t="str">
-        <v>https://doi.org/10.3390/machines13040302</v>
-      </c>
-      <c r="I9" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TEC.2020.3035165</v>
       </c>
     </row>
     <row r="10">
@@ -4589,28 +4613,25 @@
         <v>TRUE</v>
       </c>
       <c r="B10" t="str">
-        <v>90</v>
+        <v>290</v>
       </c>
       <c r="C10" t="str">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D10" t="str">
-        <v>S. H. Park and M. S. Lim*</v>
+        <v>S. H. Park, J. C. Park, S. W. Hwang, J. H. Kim, and M. S. Lim*</v>
       </c>
       <c r="E10" t="str">
-        <v>Computationally Efficient Design of 16-Poles and 24-Slots IPMSM for EV Traction Considering PWM-Induced Iron Loss Using Active Transfer Learning</v>
+        <v>Model Predictive Control for Torque Ripple Suppression Caused by Misalignment of the Gearbox</v>
       </c>
       <c r="F10" t="str">
-        <v>Mathematics, vol. 13, no. 6, pp. 915–930, Mar. 2025</v>
+        <v>IEEE Transactions on Energy Conversion, vol. 36, no. 2, pp. 1517–1527, June 2021</v>
       </c>
       <c r="G10" t="str">
-        <v>IF 2.3 · Q1 · JCR 4.2%</v>
+        <v>IF 4.614 · Q1 · JCR 14.9%</v>
       </c>
       <c r="H10" t="str">
-        <v>https://doi.org/10.3390/math13060915</v>
-      </c>
-      <c r="I10" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TEC.2021.3060536</v>
       </c>
     </row>
     <row r="11">
@@ -4618,28 +4639,25 @@
         <v>TRUE</v>
       </c>
       <c r="B11" t="str">
-        <v>100</v>
+        <v>280</v>
       </c>
       <c r="C11" t="str">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D11" t="str">
-        <v>K. S. Cha**, J. H. Kim**, S. W. Hwang, M. S. Lim*, and S. H. Park*</v>
+        <v>K. S. Cha, J. W. Chin, S. H. Park, Y. H. Jung, E. C. Lee, and M. S. Lim*</v>
       </c>
       <c r="E11" t="str">
-        <v>High-Efficiency e-Powertrain Topology by Integrating Open-End Winding and Winding Changeover for Improving Fuel Economy of Electric Vehicles</v>
+        <v>Design Method for Reducing AC Resistance of Traction Motor Using High Fill Factor Coil to Improve the Fuel Economy of eBus</v>
       </c>
       <c r="F11" t="str">
-        <v>Mathematics, vol. 12, no. 21, pp. 3415–3433, Dec. 2024</v>
+        <v>IEEE/ASME Transactions on Mechatronics, vol. 26, no. 3, pp. 1260–1270, June 2021</v>
       </c>
       <c r="G11" t="str">
-        <v>IF 2.4 · Q1 · JCR 6.8%</v>
+        <v>IF 4.943 · Q1 · JCR 5.0%</v>
       </c>
       <c r="H11" t="str">
-        <v>https://doi.org/10.3390/math12213415</v>
-      </c>
-      <c r="I11" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMECH.2021.3054798</v>
       </c>
     </row>
     <row r="12">
@@ -4647,28 +4665,25 @@
         <v>TRUE</v>
       </c>
       <c r="B12" t="str">
-        <v>110</v>
+        <v>270</v>
       </c>
       <c r="C12" t="str">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D12" t="str">
-        <v>J. H. Kim, J. Y. Ryu, S. H. Park, K. S. Cha, Y. J. Won, C. S. Park, and M. S. Lim*</v>
+        <v>H. Y. Lee, S. Y. Yoon, S. O. Kwon, J. Y. Shin, S. H. Park, and M. S. Lim*</v>
       </c>
       <c r="E12" t="str">
-        <v>Investigation on Radial Vibration of FSCW PMSM According to Pole/Slot Combination Considering Phase of Radial, Tangential Force and Moment</v>
+        <v>A Study on a Slotless Brushless DC Motor with Toroidal Winding</v>
       </c>
       <c r="F12" t="str">
-        <v>IEEE Transactions on Industry Applications, vol. 60, no. 1, pp. 439–449, Jan. 2024</v>
+        <v>Processes, vol. 9, no. 11, pp. 1881–1900, Oct. 2021</v>
       </c>
       <c r="G12" t="str">
-        <v>IF 4.079 · Q1 · JCR 24.5%</v>
+        <v>IF 2.753 · Q2</v>
       </c>
       <c r="H12" t="str">
-        <v>https://doi.org/10.1109/TIA.2023.3326425</v>
-      </c>
-      <c r="I12" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/pr9111881</v>
       </c>
     </row>
     <row r="13">
@@ -4676,28 +4691,25 @@
         <v>TRUE</v>
       </c>
       <c r="B13" t="str">
-        <v>120</v>
+        <v>260</v>
       </c>
       <c r="C13" t="str">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D13" t="str">
-        <v>S. H. Park, J. W. Chin, K. S. Cha, J. Y. Ryu, and M. S. Lim*</v>
+        <v>S. H. Park, J. W. Chin, K. S. Cha, and M. S. Lim*</v>
       </c>
       <c r="E13" t="str">
-        <v>Investigation of AC Copper Loss Considering Effect of Field and Armature Excitation on IPMSM With Hairpin Winding</v>
+        <v>Deep Transfer Learning-Based Sizing Method of Permanent Magnet Synchronous Motors Considering Axial Leakage Flux</v>
       </c>
       <c r="F13" t="str">
-        <v>IEEE Transactions on Industrial Electronics, vol. 70, no. 12, pp. 12102–12112, Dec. 2023</v>
+        <v>IEEE Transactions on Magnetics, vol. 58, no. 9, Sep. 2022</v>
       </c>
       <c r="G13" t="str">
-        <v>IF 8.236 · Q1 · JCR 2.3%</v>
+        <v>IF 1.700 · Q3</v>
       </c>
       <c r="H13" t="str">
-        <v>https://doi.org/10.1109/TIE.2023.3234154</v>
-      </c>
-      <c r="I13" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2022.3181804</v>
       </c>
     </row>
     <row r="14">
@@ -4705,28 +4717,25 @@
         <v>TRUE</v>
       </c>
       <c r="B14" t="str">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="C14" t="str">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D14" t="str">
-        <v>S. H. Park, K. O. Kim, and M. S. Lim*</v>
+        <v>J. C. Park, J. Y. Ryu, S. H. Park, and M. S. Lim*</v>
       </c>
       <c r="E14" t="str">
-        <v>Computationally Efficient Estimation of PWM-Induced Iron Loss of PMSM Using Deep Transfer Learning</v>
+        <v>Electronic Throttle Valve Modeling Considering Nonlinearity of Electrical and Mechanical Parameters Based on Experiments</v>
       </c>
       <c r="F14" t="str">
-        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
+        <v>IEEE/ASME Transactions on Mechatronics, vol. 27, no. 5, pp. 3309–3314, Oct. 2022</v>
       </c>
       <c r="G14" t="str">
-        <v>IF 1.848 · Q3</v>
+        <v>IF 5.673 · Q1 · JCR 5.0%</v>
       </c>
       <c r="H14" t="str">
-        <v>https://doi.org/10.1109/TMAG.2023.3304981</v>
-      </c>
-      <c r="I14" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMECH.2021.3123137</v>
       </c>
     </row>
     <row r="15">
@@ -4734,28 +4743,25 @@
         <v>TRUE</v>
       </c>
       <c r="B15" t="str">
-        <v>140</v>
+        <v>240</v>
       </c>
       <c r="C15" t="str">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D15" t="str">
-        <v>Y. J. Won, J. H. Kim, S. H. Park, J. H. Lee, S. M. An, D. Y. Kim, and M. S. Lim*</v>
+        <v>C. S. Park, J. H. Kim, S. H. Park, Y. D. Yoon, and M. S. Lim*</v>
       </c>
       <c r="E15" t="str">
-        <v>Transfer Learning-Based Design Method for Cogging Torque Reduction in PMSM With Step-Skew Considering 3-D Leakage Flux</v>
+        <v>Multi-physics characteristics of PMSM for compressor according to driving mode considering PWM frequency</v>
       </c>
       <c r="F15" t="str">
-        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
+        <v>IEEE Access, vol. 10, Oct. 2022</v>
       </c>
       <c r="G15" t="str">
-        <v>IF 1.848 · Q3</v>
+        <v>IF 3.367 · Q2</v>
       </c>
       <c r="H15" t="str">
-        <v>https://doi.org/10.1109/TMAG.2023.3294601</v>
-      </c>
-      <c r="I15" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/ACCESS.2022.3217779</v>
       </c>
     </row>
     <row r="16">
@@ -4763,28 +4769,25 @@
         <v>TRUE</v>
       </c>
       <c r="B16" t="str">
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="C16" t="str">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D16" t="str">
-        <v>J. C. Park, J. H. Kim, S. H. Park, K. O. Kim, M. H. Sung, and M. S. Lim</v>
+        <v>S. W. Hwang, D. K. Son, S. H. Park, G. H. Lee, Y. D. Yoon, and M. S. Lim*</v>
       </c>
       <c r="E16" t="str">
-        <v>Design Optimization Using Asymmetric Rotor in IPMSM for Torque Ripple Reduction Considering Forward and Reverse Directions</v>
+        <v>Design and Analysis of Dual Stator PMSM With Separately Controlled Dual Three-Phase Winding for eVTOL Propulsion</v>
       </c>
       <c r="F16" t="str">
-        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
+        <v>IEEE Transactions on Transportation Electrification, vol. 8, no. 4, pp. 4255–4264, Dec. 2022</v>
       </c>
       <c r="G16" t="str">
-        <v>IF 1.848 · Q3</v>
+        <v>IF 5.444 · Q1 · JCR 12.5%</v>
       </c>
       <c r="H16" t="str">
-        <v>https://doi.org/10.1109/TMAG.2023.3292295</v>
-      </c>
-      <c r="I16" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TTE.2022.3192353</v>
       </c>
     </row>
     <row r="17">
@@ -4792,28 +4795,25 @@
         <v>TRUE</v>
       </c>
       <c r="B17" t="str">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="C17" t="str">
         <v>2023</v>
       </c>
       <c r="D17" t="str">
-        <v>J. H. Lee, S. H. Park, P. J. Kim, D. H. Park, and M. S. Lim*</v>
+        <v>J. H. Kim, S. H. Park, J. Y. Ryu, and M. S. Lim*</v>
       </c>
       <c r="E17" t="str">
-        <v>Two-Dimensional FEA-Based Iron Loss Calculation Method for Linear Oscillating Actuator Considering the Circumferential Segmented Structure</v>
+        <v>Comparative Study of Vibration on 10-Pole 12-Slot and 14-Pole 12-Slot PMSM Considering Tooth Modulation Effect</v>
       </c>
       <c r="F17" t="str">
-        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
+        <v>IEEE Transactions on Industrial Electronics, vol. 70, no. 4, pp. 4007–4017, Apr. 2023</v>
       </c>
       <c r="G17" t="str">
-        <v>IF 1.848 · Q3</v>
+        <v>IF 8.236 · Q1 · JCR 2.3%</v>
       </c>
       <c r="H17" t="str">
-        <v>https://doi.org/10.1109/TMAG.2023.3275152</v>
-      </c>
-      <c r="I17" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TIE.2022.3181418</v>
       </c>
     </row>
     <row r="18">
@@ -4821,7 +4821,7 @@
         <v>TRUE</v>
       </c>
       <c r="B18" t="str">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="C18" t="str">
         <v>2023</v>
@@ -4833,7 +4833,7 @@
         <v>Effect of Electromagnetic Force Caused by PMSM on the Vibration/Noise of Reciprocating Compressors</v>
       </c>
       <c r="F18" t="str">
-        <v>IEEE Access, vol. 11, 2023</v>
+        <v>IEEE Access, vol. 11, June 2023</v>
       </c>
       <c r="G18" t="str">
         <v>IF 3.476 · Q2</v>
@@ -4841,37 +4841,31 @@
       <c r="H18" t="str">
         <v>https://doi.org/10.1109/ACCESS.2023.3283144</v>
       </c>
-      <c r="I18" t="str">
-        <v>FALSE</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
         <v>TRUE</v>
       </c>
       <c r="B19" t="str">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C19" t="str">
         <v>2023</v>
       </c>
       <c r="D19" t="str">
-        <v>J. H. Kim, S. H. Park, J. Y. Ryu, and M. S. Lim*</v>
+        <v>J. H. Lee, S. H. Park, P. J. Kim, D. H. Park, and M. S. Lim*</v>
       </c>
       <c r="E19" t="str">
-        <v>Comparative Study of Vibration on 10-Pole 12-Slot and 14-Pole 12-Slot PMSM Considering Tooth Modulation Effect</v>
+        <v>Two-Dimensional FEA-Based Iron Loss Calculation Method for Linear Oscillating Actuator Considering the Circumferential Segmented Structure</v>
       </c>
       <c r="F19" t="str">
-        <v>IEEE Transactions on Industrial Electronics, vol. 70, no. 4, pp. 4007–4017, Apr. 2023</v>
+        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
       </c>
       <c r="G19" t="str">
-        <v>IF 8.236 · Q1 · JCR 2.3%</v>
+        <v>IF 1.848 · Q3</v>
       </c>
       <c r="H19" t="str">
-        <v>https://doi.org/10.1109/TIE.2022.3181418</v>
-      </c>
-      <c r="I19" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2023.3275152</v>
       </c>
     </row>
     <row r="20">
@@ -4882,25 +4876,22 @@
         <v>190</v>
       </c>
       <c r="C20" t="str">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D20" t="str">
-        <v>C. S. Park, J. H. Kim, S. H. Park, Y. D. Yoon, and M. S. Lim*</v>
+        <v>J. C. Park, J. H. Kim, S. H. Park, K. O. Kim, M. H. Sung, and M. S. Lim*</v>
       </c>
       <c r="E20" t="str">
-        <v>Multi-physics characteristics of PMSM for compressor according to driving mode considering PWM frequency</v>
+        <v>Design Optimization Using Asymmetric Rotor in IPMSM for Torque Ripple Reduction Considering Forward and Reverse Directions</v>
       </c>
       <c r="F20" t="str">
-        <v>IEEE Access, vol. 10, 2022</v>
+        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
       </c>
       <c r="G20" t="str">
-        <v>IF 3.367 · Q2</v>
+        <v>IF 1.848 · Q3</v>
       </c>
       <c r="H20" t="str">
-        <v>https://doi.org/10.1109/ACCESS.2022.3217779</v>
-      </c>
-      <c r="I20" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2023.3292295</v>
       </c>
     </row>
     <row r="21">
@@ -4908,28 +4899,25 @@
         <v>TRUE</v>
       </c>
       <c r="B21" t="str">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C21" t="str">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D21" t="str">
-        <v>S. W. Hwang, D. K. Son, S. H. Park, G. H. Lee, Y. D. Yoon, and M. S. Lim*</v>
+        <v>Y. J. Won, J. H. Kim, S. H. Park, J. H. Lee, S. M. An, D. Y. Kim, and M. S. Lim*</v>
       </c>
       <c r="E21" t="str">
-        <v>Design and Analysis of Dual Stator PMSM With Separately Controlled Dual Three-Phase Winding for eVTOL Propulsion</v>
+        <v>Transfer Learning-Based Design Method for Cogging Torque Reduction in PMSM With Step-Skew Considering 3-D Leakage Flux</v>
       </c>
       <c r="F21" t="str">
-        <v>IEEE Transactions on Transportation Electrification, vol. 8, no. 4, pp. 4255–4264, Dec. 2022</v>
+        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
       </c>
       <c r="G21" t="str">
-        <v>IF 5.444 · Q1 · JCR 12.5%</v>
+        <v>IF 1.848 · Q3</v>
       </c>
       <c r="H21" t="str">
-        <v>https://doi.org/10.1109/TTE.2022.3192353</v>
-      </c>
-      <c r="I21" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2023.3294601</v>
       </c>
     </row>
     <row r="22">
@@ -4937,28 +4925,25 @@
         <v>TRUE</v>
       </c>
       <c r="B22" t="str">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C22" t="str">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D22" t="str">
-        <v>J. C. Park, J. Y. Ryu, S. H. Park, and M. S. Lim*</v>
+        <v>S. H. Park, K. O. Kim, and M. S. Lim*</v>
       </c>
       <c r="E22" t="str">
-        <v>Electronic Throttle Valve Modeling Considering Nonlinearity of Electrical and Mechanical Parameters Based on Experiments</v>
+        <v>Computationally Efficient Estimation of PWM-Induced Iron Loss of PMSM Using Deep Transfer Learning</v>
       </c>
       <c r="F22" t="str">
-        <v>IEEE/ASME Transactions on Mechatronics, vol. 27, no. 5, pp. 3309–3314, Oct. 2022</v>
+        <v>IEEE Transactions on Magnetics, vol. 59, no. 11, Nov. 2023</v>
       </c>
       <c r="G22" t="str">
-        <v>IF 5.673 · Q1 · JCR 5.0%</v>
+        <v>IF 1.848 · Q3</v>
       </c>
       <c r="H22" t="str">
-        <v>https://doi.org/10.1109/TMECH.2021.3123137</v>
-      </c>
-      <c r="I22" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2023.3304981</v>
       </c>
     </row>
     <row r="23">
@@ -4966,28 +4951,25 @@
         <v>TRUE</v>
       </c>
       <c r="B23" t="str">
-        <v>220</v>
+        <v>160</v>
       </c>
       <c r="C23" t="str">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D23" t="str">
-        <v>S. H. Park, J. W. Chin, K. S. Cha, and M. S. Lim*</v>
+        <v>S. H. Park, J. W. Chin, K. S. Cha, J. Y. Ryu, and M. S. Lim*</v>
       </c>
       <c r="E23" t="str">
-        <v>Deep Transfer Learning-Based Sizing Method of Permanent Magnet Synchronous Motors Considering Axial Leakage Flux</v>
+        <v>Investigation of AC Copper Loss Considering Effect of Field and Armature Excitation on IPMSM With Hairpin Winding</v>
       </c>
       <c r="F23" t="str">
-        <v>IEEE Transactions on Magnetics, vol. 58, no. 9, Sep. 2022</v>
+        <v>IEEE Transactions on Industrial Electronics, vol. 70, no. 12, pp. 12102–12112, Dec. 2023</v>
       </c>
       <c r="G23" t="str">
-        <v>IF 1.700 · Q3</v>
+        <v>IF 8.236 · Q1 · JCR 2.3%</v>
       </c>
       <c r="H23" t="str">
-        <v>https://doi.org/10.1109/TMAG.2022.3181804</v>
-      </c>
-      <c r="I23" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TIE.2023.3234154</v>
       </c>
     </row>
     <row r="24">
@@ -4995,28 +4977,25 @@
         <v>TRUE</v>
       </c>
       <c r="B24" t="str">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="C24" t="str">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D24" t="str">
-        <v>H. Y. Lee, S. Y. Yoon, S. O. Kwon, J. Y. Shin, S. H. Park, and M. S. Lim*</v>
+        <v>J. H. Kim, J. Y. Ryu, S. H. Park, K. S. Cha, Y. J. Won, C. S. Park, and M. S. Lim*</v>
       </c>
       <c r="E24" t="str">
-        <v>A Study on a Slotless Brushless DC Motor with Toroidal Winding</v>
+        <v>Investigation on Radial Vibration of FSCW PMSM According to Pole/Slot Combination Considering Phase of Radial, Tangential Force and Moment</v>
       </c>
       <c r="F24" t="str">
-        <v>Processes, vol. 9, no. 11, pp. 1881–1900, Oct. 2021</v>
+        <v>IEEE Transactions on Industry Applications, vol. 60, no. 1, pp. 439–449, Jan. 2024</v>
       </c>
       <c r="G24" t="str">
-        <v>IF 2.753 · Q2</v>
+        <v>IF 4.079 · Q1 · JCR 24.5%</v>
       </c>
       <c r="H24" t="str">
-        <v>https://doi.org/10.3390/pr9111881</v>
-      </c>
-      <c r="I24" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TIA.2023.3326425</v>
       </c>
     </row>
     <row r="25">
@@ -5024,28 +5003,25 @@
         <v>TRUE</v>
       </c>
       <c r="B25" t="str">
-        <v>240</v>
+        <v>140</v>
       </c>
       <c r="C25" t="str">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D25" t="str">
-        <v>K. S. Cha, J. W. Chin, S. H. Park, Y. H. Jung, E. C. Lee, and M. S. Lim*</v>
+        <v>K. S. Cha**, J. H. Kim**, S. W. Hwang, M. S. Lim*, and S. H. Park*</v>
       </c>
       <c r="E25" t="str">
-        <v>Design Method for Reducing AC Resistance of Traction Motor Using High Fill Factor Coil to Improve the Fuel Economy of eBus</v>
+        <v>High-Efficiency e-Powertrain Topology by Integrating Open-End Winding and Winding Changeover for Improving Fuel Economy of Electric Vehicles</v>
       </c>
       <c r="F25" t="str">
-        <v>IEEE/ASME Transactions on Mechatronics, vol. 26, no. 3, pp. 1260–1270, June 2021</v>
+        <v>Mathematics, vol. 12, no. 21, pp. 3415–3433, Dec. 2024</v>
       </c>
       <c r="G25" t="str">
-        <v>IF 4.943 · Q1 · JCR 13.3%</v>
+        <v>IF 2.4 · Q1 · JCR 6.8%</v>
       </c>
       <c r="H25" t="str">
-        <v>https://doi.org/10.1109/TMECH.2021.3054798</v>
-      </c>
-      <c r="I25" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/math12213415</v>
       </c>
     </row>
     <row r="26">
@@ -5053,28 +5029,25 @@
         <v>TRUE</v>
       </c>
       <c r="B26" t="str">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="C26" t="str">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D26" t="str">
-        <v>S. H. Park, J. C. Park, S. W. Hwang, J. H. Kim, and M. S. Lim*</v>
+        <v>S. H. Park and M. S. Lim*</v>
       </c>
       <c r="E26" t="str">
-        <v>Model Predictive Control for Torque Ripple Suppression Caused by Misalignment of the Gearbox</v>
+        <v>Computationally Efficient Design of 16-Poles and 24-Slots IPMSM for EV Traction Considering PWM-Induced Iron Loss Using Active Transfer Learning</v>
       </c>
       <c r="F26" t="str">
-        <v>IEEE Transactions on Energy Conversion, vol. 36, no. 2, pp. 1517–1527, June 2021</v>
+        <v>Mathematics, vol. 13, no. 6, pp. 915–930, Mar. 2025</v>
       </c>
       <c r="G26" t="str">
-        <v>IF 4.614 · Q1 · JCR 14.9%</v>
+        <v>IF 2.3 · Q1 · JCR 4.2%</v>
       </c>
       <c r="H26" t="str">
-        <v>https://doi.org/10.1109/TEC.2021.3060536</v>
-      </c>
-      <c r="I26" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/math13060915</v>
       </c>
     </row>
     <row r="27">
@@ -5082,28 +5055,25 @@
         <v>TRUE</v>
       </c>
       <c r="B27" t="str">
-        <v>260</v>
+        <v>120</v>
       </c>
       <c r="C27" t="str">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D27" t="str">
-        <v>J. W. Chin, K. S. Cha, M. R. Park, S. H. Park, E. C. Lee, and M. S. Lim*</v>
+        <v>M. H. Sung**, S. H. Park**, K. S. Cha, J. H. Sim, and M. S. Lim*</v>
       </c>
       <c r="E27" t="str">
-        <v>High Efficiency PMSM With High Slot Fill Factor Coil for Heavy-Duty EV Traction Considering AC Resistance</v>
+        <v>Deep Transfer Learning-Based Performance Prediction Considering 3-D Flux in Outer Rotor Interior Permanent Magnet Synchronous Motors</v>
       </c>
       <c r="F27" t="str">
-        <v>IEEE Transactions on Energy Conversion, vol. 36, no. 2, pp. 883–894, June 2021</v>
+        <v>Machines, vol. 13, no. 4, pp. 302–313, Apr. 2025</v>
       </c>
       <c r="G27" t="str">
-        <v>IF 4.614 · Q1 · JCR 14.9%</v>
+        <v>IF 2.1 · Q2</v>
       </c>
       <c r="H27" t="str">
-        <v>https://doi.org/10.1109/TEC.2020.3035165</v>
-      </c>
-      <c r="I27" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/machines13040302</v>
       </c>
     </row>
     <row r="28">
@@ -5111,28 +5081,25 @@
         <v>TRUE</v>
       </c>
       <c r="B28" t="str">
-        <v>270</v>
+        <v>110</v>
       </c>
       <c r="C28" t="str">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D28" t="str">
-        <v>S. W. Hwang, J. Y. Ryu, J. W. Chin, S. H. Park, D. K. Kim, and M. S. Lim*</v>
+        <v>K. S. Cha**, Y. H. Jung**, S. H. Park*, and M. R. Park*</v>
       </c>
       <c r="E28" t="str">
-        <v>Coupled Electromagnetic-Thermal Analysis for Predicting Traction Motor Characteristics According to Electric Vehicle Driving Cycle</v>
+        <v>Optimal Design Considering AC Copper Loss of Traction Motor Applied HSFF Coil for Improving Electric Bus Fuel Economy</v>
       </c>
       <c r="F28" t="str">
-        <v>IEEE Transactions on Vehicular Technology, vol. 70, no. 5, pp. 4262–4272, May 2021</v>
+        <v>Mathematics, vol. 13, no. 9, pp. 1509–1528, May 2025</v>
       </c>
       <c r="G28" t="str">
-        <v>IF 5.379 · Q1 · JCR 12.6%</v>
+        <v>IF 2.3 · Q1 · JCR 4.2%</v>
       </c>
       <c r="H28" t="str">
-        <v>https://doi.org/10.1109/TVT.2021.3071943</v>
-      </c>
-      <c r="I28" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/math13091509</v>
       </c>
     </row>
     <row r="29">
@@ -5140,28 +5107,25 @@
         <v>TRUE</v>
       </c>
       <c r="B29" t="str">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="C29" t="str">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D29" t="str">
-        <v>S. H. Park, E. C. Lee, G. J. Lee, S. O. Kwon, and M. S. Lim*</v>
+        <v>Y. H. Jung**, D. M. Kim**, K. S. Cha, S. H. Park*, and M. R. Park*</v>
       </c>
       <c r="E29" t="str">
-        <v>Effect of Pole and Slot Combination on the AC Joule Loss of Outer-Rotor Permanent Magnet Synchronous Motors Using a High Fill Factor Machined Coil</v>
+        <v>Vibration Reduction of Permanent Magnet Synchronous Motors by Four-Layer Winding: Mathematical Modeling and Experimental Validation</v>
       </c>
       <c r="F29" t="str">
-        <v>Energies, vol. 14, no. 11, pp. 3073–3083, May 2021</v>
+        <v>Mathematics, vol. 13, no. 9, pp. 1603–1621, May 2025</v>
       </c>
       <c r="G29" t="str">
-        <v>IF 2.702 · Q3</v>
+        <v>IF 2.3 · Q1 · JCR 4.2%</v>
       </c>
       <c r="H29" t="str">
-        <v>https://doi.org/10.3390/en14113073</v>
-      </c>
-      <c r="I29" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/math13101603</v>
       </c>
     </row>
     <row r="30">
@@ -5169,28 +5133,25 @@
         <v>TRUE</v>
       </c>
       <c r="B30" t="str">
-        <v>290</v>
+        <v>90</v>
       </c>
       <c r="C30" t="str">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="D30" t="str">
-        <v>J. C. Park, S. H. Park, J. H. Kim, S. G. Lee, G. H. Lee, and M. S. Lim*</v>
+        <v>S. Khalid, J. W. Song, M. H. Yazdani, M. U. Elahi, S. H. Park, H. S. Kim*, Y. G. Yoon, and J. S. Lee</v>
       </c>
       <c r="E30" t="str">
-        <v>Diagnosis and Robust Design Optimization of SPMSM Considering Back EMF and Cogging Torque due to Static Eccentricity</v>
+        <v>Advances in prognostics and health management of light emitting diodes: A comprehensive review</v>
       </c>
       <c r="F30" t="str">
-        <v>Energies, vol. 14, no. 10, pp. 2900–2918, May 2021</v>
+        <v>Journal of Computational Design and Engineering, vol. 12, no. 9, pp. 184–203, Sept. 2025</v>
       </c>
       <c r="G30" t="str">
-        <v>IF 2.702 · Q3</v>
+        <v>IF 4.8 · Q1 · JCR 11.3%</v>
       </c>
       <c r="H30" t="str">
-        <v>https://doi.org/10.3390/en14102900</v>
-      </c>
-      <c r="I30" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1093/jcde/qwaf090</v>
       </c>
     </row>
     <row r="31">
@@ -5198,28 +5159,25 @@
         <v>TRUE</v>
       </c>
       <c r="B31" t="str">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="C31" t="str">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="D31" t="str">
-        <v>S. H. Park, E. C. Lee, J. C. Park, S. W. Hwang, and M. S. Lim*</v>
+        <v>J. H. Lee, S. H. Park, D. H. Park, J. H. Jeong, and M. S. Lim*</v>
       </c>
       <c r="E31" t="str">
-        <v>Prediction of Mechanical Loss for High-Power Density PMSM Considering Eddy Current Loss of PMs and Conductors</v>
+        <v>Deep Transfer Learning-Based Demagnetization Analysis for Linear Oscillating Actuator Considering Circumferential Segmented Structure</v>
       </c>
       <c r="F31" t="str">
-        <v>IEEE Transactions on Magnetics, vol. 57, no. 2, Feb. 2021</v>
+        <v>IEEE Transactions on Industry Applications, vol. 62, no. 1, pp. 821–829, Jan. 2026</v>
       </c>
       <c r="G31" t="str">
-        <v>IF 1.651 · Q3</v>
+        <v>IF 4.2 · Q1 · JCR 13.0%</v>
       </c>
       <c r="H31" t="str">
-        <v>https://doi.org/10.1109/TMAG.2020.3007439</v>
-      </c>
-      <c r="I31" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TIA.2025.3585098</v>
       </c>
     </row>
     <row r="32">
@@ -5227,28 +5185,25 @@
         <v>TRUE</v>
       </c>
       <c r="B32" t="str">
-        <v>310</v>
+        <v>70</v>
       </c>
       <c r="C32" t="str">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="D32" t="str">
-        <v>S. H. Park, J. C. Park, H. Y. Lee, S. O. Kwon, and M. S. Lim*</v>
+        <v>J. H. Kim, Y. J. Won, S. H. Park, and M. S. Lim*</v>
       </c>
       <c r="E32" t="str">
-        <v>Design of High-Bandwidth Motor System Considering Electrical and Mechanical Time Constant</v>
+        <v>Effect of Manufacturing Tolerances and Magnetic Anisotropy of Electrical Steel on Surface-Mounted Permanent Magnet Synchronous Motor Cogging Torque</v>
       </c>
       <c r="F32" t="str">
-        <v>IEEE Transactions on Industry Applications, vol. 56, no. 5, pp. 4738–4747, Sep. 2020</v>
+        <v>Mathematics, vol. 14, no. 4, pp. 650–665, Feb. 2026</v>
       </c>
       <c r="G32" t="str">
-        <v>IF 2.743 · Q1 · JCR 15.7%</v>
+        <v>IF 2.2 · Q1 · JCR 6.0%</v>
       </c>
       <c r="H32" t="str">
-        <v>https://doi.org/10.1109/TIA.2020.2998674</v>
-      </c>
-      <c r="I32" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.3390/math14040650</v>
       </c>
     </row>
     <row r="33">
@@ -5256,28 +5211,25 @@
         <v>TRUE</v>
       </c>
       <c r="B33" t="str">
-        <v>320</v>
+        <v>60</v>
       </c>
       <c r="C33" t="str">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="D33" t="str">
-        <v>S. H. Park, J. C. Park, S. W. Hwang, J. H. Kim, H. J. Park, and M. S. Lim*</v>
+        <v>J. K. Ryu, C. W. Kim, S. W. Jeong, M. R. Park*, and S. H. Park*</v>
       </c>
       <c r="E33" t="str">
-        <v>Suppression of Torque Ripple Caused by Misalignment of the Gearbox by Using Harmonic Current Injection Method</v>
+        <v>Efficient multi-objective design optimization of axial-flux permanent magnet machines for drone propulsion system using multi-fidelity gaussian process</v>
       </c>
       <c r="F33" t="str">
-        <v>IEEE/ASME Transactions on Mechatronics, vol. 25, no. 4, pp. 1990–1999, Aug. 2020</v>
+        <v>Structural and Multidisciplinary Optimization, vol. 69, no. 5, Apr. 2026</v>
       </c>
       <c r="G33" t="str">
-        <v>IF 4.943 · Q1 · JCR 5.0%</v>
+        <v>IF 4.0 · Q1 · JCR 16.5%</v>
       </c>
       <c r="H33" t="str">
-        <v>https://doi.org/10.1109/TMECH.2020.2999379</v>
-      </c>
-      <c r="I33" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1007/s00158-026-04316-8</v>
       </c>
     </row>
     <row r="34">
@@ -5285,28 +5237,25 @@
         <v>TRUE</v>
       </c>
       <c r="B34" t="str">
-        <v>330</v>
+        <v>50</v>
       </c>
       <c r="C34" t="str">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="D34" t="str">
-        <v>G. J. Lee, H. Y. Lee, E. C. Lee, S. H. Park, S. O. Kwon, H. S. Choi*, and J. H. Seo</v>
+        <v>S. H. Park, D. H. Ko, S. G. Lee, J. C. Park, and M. R. Park*</v>
       </c>
       <c r="E34" t="str">
-        <v>Analysis of AC Resistance according to Coil Shape of an Interior-Permanent Magnet Motor</v>
+        <v>Robust Design Optimization of SPMSM based on Manufacturing Uncertainty Analysis of Prototype</v>
       </c>
       <c r="F34" t="str">
-        <v>The Transactions of the Korean Institute of Electrical Engineers, vol. 69, no. 5, pp. 671–676, May 2020</v>
+        <v>IEEE Transactions on Magnetics, vol. 62, no. 7, Jul. 2026</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>IF 2.1 · Q3</v>
       </c>
       <c r="H34" t="str">
-        <v>https://doi.org/10.5370/KIEE.2020.69.5.671</v>
-      </c>
-      <c r="I34" t="str">
-        <v>FALSE</v>
+        <v>https://doi.org/10.1109/TMAG.2025.3616812</v>
       </c>
     </row>
     <row r="35">
@@ -5314,40 +5263,121 @@
         <v>TRUE</v>
       </c>
       <c r="B35" t="str">
-        <v>340</v>
+        <v>40</v>
       </c>
       <c r="C35" t="str">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="D35" t="str">
-        <v>S. H. Park, J. C. Park, J. W. Chin, H. J. Park, S. O. Kwon, S. I. Kim, and M. S. Lim*</v>
+        <v>Y. M. Lee, D. H. Ko, S. Yoon, J. Cho, S. H. Park*, and M. R. Park*</v>
       </c>
       <c r="E35" t="str">
-        <v>Design of Surface-mounted Permanent Magnet Synchronous Motor using Electromagnetic and Thermal Analysis</v>
+        <v>Characteristics Estimation and Design of SPMSM using Analytic Method-based Transfer Learning</v>
       </c>
       <c r="F35" t="str">
-        <v>Journal of Magnetics, vol. 24, no. 4, pp. 606–615, Dec. 2019</v>
+        <v>IEEE Transactions on Magnetics, vol. 62, no. 7, Jul. 2026</v>
       </c>
       <c r="G35" t="str">
-        <v>IF 0.628 · Q4</v>
+        <v>IF 2.1 · Q3</v>
       </c>
       <c r="H35" t="str">
-        <v>https://doi.org/10.4283/JMAG.2019.24.4.606</v>
-      </c>
-      <c r="I35" t="str">
+        <v>https://doi.org/10.1109/TMAG.2025.3640767</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B36" t="str">
+        <v>30</v>
+      </c>
+      <c r="C36" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D36" t="str">
+        <v>K. S. Cha**, S. H. Park**, and Y. H. Jung*</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Design of WFSM using Sizing Method Combining 2D Equivalent Magnetic Circuit Considering Nonlinear Characteristics</v>
+      </c>
+      <c r="F36" t="str">
+        <v>IEEE Transactions on Magnetics, vol. 62, no. 7, Jul. 2026</v>
+      </c>
+      <c r="G36" t="str">
+        <v>IF 2.1 · Q3</v>
+      </c>
+      <c r="H36" t="str">
+        <v>https://doi.org/10.1109/TMAG.2025.3624623</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B37" t="str">
+        <v>20</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D37" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Iron Loss Calculation Method Considering Slot Harmonic Components for Induction Motor Using Virtual Blocked Rotor and Transfer Learning</v>
+      </c>
+      <c r="F37" t="str">
+        <v>IEEE Transactions on Industry Applications, Early Access, 2026</v>
+      </c>
+      <c r="G37" t="str">
+        <v>IF 4.5 · Q1 · JCR 14.8%</v>
+      </c>
+      <c r="H37" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://doi.org/10.1109/TIA.2026.3721841_x000d_
+</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B38" t="str">
+        <v>10</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D38" t="str">
+        <v>H. S. Kim**, S. H. Park**, Y. M. Lee, and M. R. Park*</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Transfer Learning-Assisted Analytical Quasi-3D Surrogate Modeling for Electromagnetic Performance Prediction of AFPMs Considering Eccentricity</v>
+      </c>
+      <c r="F38" t="str">
+        <v>IEEE Transactions on Magnetics, Early Access, 2026</v>
+      </c>
+      <c r="G38" t="str">
+        <v>IF 1.9 · Q3</v>
+      </c>
+      <c r="H38" t="str">
+        <v>https://doi.org/10.1109/TMAG.2026.3701418</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
         <v>FALSE</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H39"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I44"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5378,30 +5408,31 @@
         <v>notes</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>430</v>
       </c>
       <c r="C2" t="str">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="D2" t="str">
-        <v>(예: 홍길동, 박수환)</v>
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
       </c>
       <c r="E2" t="str">
-        <v>(발표 논문 제목)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>(학술대회명, 예: KSAE 춘계학술대회)</v>
+        <v>Design of High Bandwidth Motor System Considering Electrical and Mechanical Time Constants</v>
+      </c>
+      <c r="F2" t="str" xml:space="preserve">
+        <v xml:space="preserve">IEEE Energy Conversion Congress &amp;
+ Expo 2019 (ECCE 2019)</v>
       </c>
       <c r="G2" t="str">
-        <v>(예: 제주)</v>
+        <v>Baltimore, USA</v>
       </c>
       <c r="H2" t="str">
-        <v>2025.05</v>
+        <v>2019.09</v>
       </c>
       <c r="I2" t="str">
         <v>발표 목록 데이터 입력 필요 — 원본 디자인은 placeholder</v>
@@ -5409,28 +5440,28 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="B3" t="str">
-        <v>20</v>
+        <v>420</v>
       </c>
       <c r="C3" t="str">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="D3" t="str">
-        <v>김찬우, 박수환</v>
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
       </c>
       <c r="E3" t="str">
-        <v>[샘플] IPMSM의 PWM 고조파를 고려한 철손 예측 기법</v>
+        <v>Design of PMSM for EV Traction using MSO Coil Considering AC Resistance According to Current Density and Parallel Circuit</v>
       </c>
       <c r="F3" t="str">
-        <v>한국자동차공학회 춘계학술대회</v>
+        <v>IEEE Vehicular Power and Propulsion Conference 2019 (VPPC 2019)</v>
       </c>
       <c r="G3" t="str">
-        <v>제주</v>
+        <v>Hanoi, Vietnam</v>
       </c>
       <c r="H3" t="str">
-        <v>2025.05</v>
+        <v>2019.1</v>
       </c>
       <c r="I3" t="str">
         <v>샘플 행 — 실제 발표로 교체할 것</v>
@@ -5438,43 +5469,1084 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="B4" t="str">
-        <v>30</v>
+        <v>410</v>
       </c>
       <c r="C4" t="str">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="D4" t="str">
-        <v>유재경, 박수환</v>
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
       </c>
       <c r="E4" t="str">
-        <v>[샘플] 드론용 축방향 자속 전동기의 다중충실도 최적설계</v>
+        <v>AC Resistance Reduction Design of Traction Motor for High Energy Efficiency of Electric Vehicle</v>
       </c>
       <c r="F4" t="str">
-        <v>대한전기학회 하계학술대회</v>
+        <v>IEEE Vehicular Power and Propulsion Conference 2019 (VPPC 2019)</v>
       </c>
       <c r="G4" t="str">
-        <v>부산</v>
+        <v>Hanoi, Vietnam</v>
       </c>
       <c r="H4" t="str">
-        <v>2024.07</v>
+        <v>2019.1</v>
       </c>
       <c r="I4" t="str">
         <v>샘플 행 — 실제 발표로 교체할 것</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B5" t="str">
+        <v>400</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2020</v>
+      </c>
+      <c r="D5" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Suppression of Torque Ripple Caused by Misalignment of the Gearbox by Using Harmonic Current Injection Method</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2020 IEEE/ASME International Conference on Advanced Intelligent Mechatronics (AIM 2020)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Boston, USA</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2020.07</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B6" t="str">
+        <v>390</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2020</v>
+      </c>
+      <c r="D6" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Effect of Pole and Slot Combination on the AC Joule Loss of Open-Slot PMSM using MSO Coil</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2020 Conference on Electromagnetic Field Computation (CEFC 2020)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Pisa, Italy</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2020.11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B7" t="str">
+        <v>380</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2020</v>
+      </c>
+      <c r="D7" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Analysis of 1kW Drone Drive Motor Characteristics with Cu and Al MSO Coil</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2020 Conference on Electromagnetic Field Computation (CEFC 2020)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Pisa, Italy</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2020.11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B8" t="str">
+        <v>370</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2020</v>
+      </c>
+      <c r="D8" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Analytic Method for Magnetic Field Computation of Surface Mounted Permanent Magnet Synchronous Machines with Cycloid Shaped Magnet</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2020 Conference on Electromagnetic Field Computation (CEFC 2020)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Pisa, Italy</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2020.11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B9" t="str">
+        <v>360</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2021</v>
+      </c>
+      <c r="D9" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Design Optimization for Torque Ripple Reduction using an Asymmetric Rotor in IPMSM Considering the Forward and Reverse Directions</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2021 International Conference on Magnetics (INTERMAG 2021)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Lyon, France</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2021.04</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B10" t="str">
+        <v>350</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2021</v>
+      </c>
+      <c r="D10" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Reduction of IPMSM with Asymmetric Rotor Shape under Certain Load Condition</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2021 International Conference on Magnetics (INTERMAG 2021)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Lyon, France</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2021.04</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B11" t="str">
+        <v>340</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2021</v>
+      </c>
+      <c r="D11" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Characteristics Analysis of IPMSM for EV Traction Considering the Effect of Field and Armature Excitations on AC Copper Loss</v>
+      </c>
+      <c r="F11" t="str" xml:space="preserve">
+        <v xml:space="preserve">IEEE Energy Conversion Congress &amp;
+ Expo 2021 (ECCE 2021)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Vancouver, Canada</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2021.10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B12" t="str">
+        <v>330</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2021</v>
+      </c>
+      <c r="D12" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Temperature Prediction of Ultra-High-Speed SPMSM for FCEV Air Compressor Considering PWM Current Harmonics</v>
+      </c>
+      <c r="F12" t="str">
+        <v>IEEE Vehicular Power and Propulsion Conference 2021 (VPPC 2021)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Gijon, Spain</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2021.10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B13" t="str">
+        <v>320</v>
+      </c>
+      <c r="C13" t="str">
+        <v>2021</v>
+      </c>
+      <c r="D13" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Open-End Winding Permanent Magnet Synchronous Machine With Winding Connection Change Method for High Efficiency EV Traction</v>
+      </c>
+      <c r="F13" t="str">
+        <v>IEEE Vehicular Power and Propulsion Conference 2021 (VPPC 2021)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Gijon, Spain</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2021.10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B14" t="str">
+        <v>310</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2022</v>
+      </c>
+      <c r="D14" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Deep Learning-Based Sizing Method of SPMSM Considering Axial Leakage Flux</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2021 International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2021)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Cancun, Mexico</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2022.01</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B15" t="str">
+        <v>300</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2023</v>
+      </c>
+      <c r="D15" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Computationally Efficient Estimation of PWM-induced Iron Loss of PMSM using Deep Transfer Learning</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2023 International Conference on Magnetics (INTERMAG 2023)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Sendai, Japan</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2023.05</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B16" t="str">
+        <v>290</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2023</v>
+      </c>
+      <c r="D16" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Transfer Learning-Based Design Method for Cogging Torque Reduction in PMSM with Step-Skew Considering 3-D Leakage Flux</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2023 International Conference on Magnetics (INTERMAG 2023)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Sendai, Japan</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2023.05</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B17" t="str">
+        <v>280</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2023</v>
+      </c>
+      <c r="D17" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2-D FEA-Based Iron Loss Calculation Method for Linear Oscillating Actuator Considering the Circumferential Segmented Structure</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2023 International Conference on Magnetics (INTERMAG 2023)</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Sendai, Japan</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2023.05</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B18" t="str">
+        <v>270</v>
+      </c>
+      <c r="C18" t="str">
+        <v>2024</v>
+      </c>
+      <c r="D18" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Suppression of Vibration in PMSM Caused by Time-Varying Load for Reciprocating Compressor</v>
+      </c>
+      <c r="F18" t="str">
+        <v>26th International Conference on Electrical Machines 2024 (ICEM 2024)</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Torino, Italy</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2024.09</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B19" t="str">
+        <v>260</v>
+      </c>
+      <c r="C19" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D19" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Design Optimization of Single-Phase Linear Oscillating Actuator Considering Effect of Detent Force on Mechanical Resonance in Linear Compressor</v>
+      </c>
+      <c r="F19" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B20" t="str">
+        <v>250</v>
+      </c>
+      <c r="C20" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D20" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E20" t="str">
+        <v>A Comparative Study of Dual Mover and Dual Stator Linear Oscillating Actuator Considering Mechanical Resonance in Linear Compressor</v>
+      </c>
+      <c r="F20" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B21" t="str">
+        <v>240</v>
+      </c>
+      <c r="C21" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D21" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Analysis of 2-D FEA Methods for Linear Oscillating Actuators Considering the Segmented Structure</v>
+      </c>
+      <c r="F21" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H21" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B22" t="str">
+        <v>230</v>
+      </c>
+      <c r="C22" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D22" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Integration of Coil Winding Process into Linear Oscillating Actuators Design</v>
+      </c>
+      <c r="F22" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B23" t="str">
+        <v>220</v>
+      </c>
+      <c r="C23" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D23" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E23" t="str">
+        <v>A Comparative Study of Multi-Objective Optimization in Linear Oscillating Actuators</v>
+      </c>
+      <c r="F23" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H23" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B24" t="str">
+        <v>210</v>
+      </c>
+      <c r="C24" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D24" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Performances Analysis of Linear Oscillating Actuator with Dual Stator Topology</v>
+      </c>
+      <c r="F24" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H24" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B25" t="str">
+        <v>200</v>
+      </c>
+      <c r="C25" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D25" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Improved Loss Analysis Method Considering Core Anisotropy and AC Copper Loss in Linear Oscillating Actuator</v>
+      </c>
+      <c r="F25" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H25" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B26" t="str">
+        <v>190</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D26" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Comparison of Prediction Accuracy between Kriging and Deep Neural Network Surrogate Models for Design Optimization of Linear Oscillating Actuators</v>
+      </c>
+      <c r="F26" t="str">
+        <v>The 15th International Symposium on Linear Drives for Industry Applications (LDIA 2025)</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Daejeon, Republic of Korea</v>
+      </c>
+      <c r="H26" t="str">
+        <v>2025.05</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B27" t="str">
+        <v>180</v>
+      </c>
+      <c r="C27" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D27" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Computationally Efficient Conductor Design for WFSM with Hairpin Windings Considering AC Ohmic Loss</v>
+      </c>
+      <c r="F27" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H27" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B28" t="str">
+        <v>170</v>
+      </c>
+      <c r="C28" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D28" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Design of WFSM using Sizing Method Combining 2D Equivalent Magnetic Circuit considering Nonlinear Characteristics</v>
+      </c>
+      <c r="F28" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H28" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B29" t="str">
+        <v>160</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D29" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Robust Design Optimization of SPMSM based on Manufacturing Uncertainty Analysis of Prototype</v>
+      </c>
+      <c r="F29" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H29" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B30" t="str">
+        <v>150</v>
+      </c>
+      <c r="C30" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D30" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Computationally Efficient Surrogate Modeling of PWM-Induced Iron Loss for Axial Flux Permanent Magnet Synchronous Motors Using Deep Transfer Learning</v>
+      </c>
+      <c r="F30" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H30" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B31" t="str">
+        <v>140</v>
+      </c>
+      <c r="C31" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D31" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Efficient Prediction of Electromagnetic Excitation Force for SPMSM Using Analytical Model-Based Deep Transfer Learning Considering Axial Leakage Flux</v>
+      </c>
+      <c r="F31" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H31" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B32" t="str">
+        <v>130</v>
+      </c>
+      <c r="C32" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D32" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Efficient Analysis of Efficiency Map for Externally Excited Synchronous Motors Using Equivalent Magnetic Circuit-Based Deep Transfer Learning</v>
+      </c>
+      <c r="F32" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H32" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B33" t="str">
+        <v>120</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D33" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Characteristics Estimation and Design of SPMSM using Analytic Method-based Transfer Learning</v>
+      </c>
+      <c r="F33" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H33" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B34" t="str">
+        <v>110</v>
+      </c>
+      <c r="C34" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D34" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Effect of Magnetic Anisotropy Property of Non-Oriented Electrical Steel on SPMSM Cogging Torque</v>
+      </c>
+      <c r="F34" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H34" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B35" t="str">
+        <v>100</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D35" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Analytic Estimation and Verification of Cogging Torque in SPMSM with Manufacturing Tolerance of Segmented Core</v>
+      </c>
+      <c r="F35" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H35" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B36" t="str">
+        <v>90</v>
+      </c>
+      <c r="C36" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D36" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Comparative Study of Kriging and Deep Neural Network as Surrogate Models for Performance Prediction of PMSM</v>
+      </c>
+      <c r="F36" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H36" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B37" t="str">
+        <v>80</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D37" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Computationally Efficient Sensitivity Analysis for robustness of Electric Motor considering Manufacturing Uncertainty</v>
+      </c>
+      <c r="F37" t="str">
+        <v>25th International Conference on the Computation of Electromagnetic Fields (COMPUMAG 2025)</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Naples, Italy</v>
+      </c>
+      <c r="H37" t="str">
+        <v>2025.06</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B38" t="str">
+        <v>70</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D38" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Virtual Vibration Sensor Calibration Based on VAE-Based Transfer Learning for Predicting Low Frequency Vibration on Permanent Magnet Synchronous Motors</v>
+      </c>
+      <c r="F38" t="str">
+        <v>31st International Congress on Sound and Vibration (ICSV 31)</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Incheon, Republic of Korea</v>
+      </c>
+      <c r="H38" t="str">
+        <v>2025.07</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B39" t="str">
+        <v>60</v>
+      </c>
+      <c r="C39" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D39" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Computationally Efficient Prediction of Electromagnetic Excitation Force in SPMSM Considering Axial Leakage Flux via Space Harmonic Analysis-Based Deep Transfer Learning</v>
+      </c>
+      <c r="F39" t="str">
+        <v>27th International Conference on Electrical Machines 2024 (ICEM 2026)</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Funchal, Portugal</v>
+      </c>
+      <c r="H39" t="str">
+        <v>2026.09</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B40" t="str">
+        <v>50</v>
+      </c>
+      <c r="C40" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D40" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Data-Driven Multi-State Flux Model for Enhanced Static Eccentricity Diagnosis of IPMSMs</v>
+      </c>
+      <c r="F40" t="str">
+        <v>27th International Conference on Electrical Machines 2024 (ICEM 2026)</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Funchal, Portugal</v>
+      </c>
+      <c r="H40" t="str">
+        <v>2026.09</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B41" t="str">
+        <v>40</v>
+      </c>
+      <c r="C41" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D41" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Analysis of IPMSM for Direct-Drive Compander Considering Temperature-Gradient in Axial Direction</v>
+      </c>
+      <c r="F41" t="str">
+        <v>27th International Conference on Electrical Machines 2024 (ICEM 2026)</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Funchal, Portugal</v>
+      </c>
+      <c r="H41" t="str">
+        <v>2026.09</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B42" t="str">
+        <v>30</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D42" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E42" t="str">
+        <v>EMC-Based Geometric Scaling Method for Axial Flux Permanent Magnet Motors</v>
+      </c>
+      <c r="F42" t="str">
+        <v>27th International Conference on Electrical Machines 2024 (ICEM 2026)</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Funchal, Portugal</v>
+      </c>
+      <c r="H42" t="str">
+        <v>2026.09</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B43" t="str">
+        <v>20</v>
+      </c>
+      <c r="C43" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D43" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E43" t="str">
+        <v>A Scaling Framework for Efficient Design Optimization of IPMSM for EV Traction</v>
+      </c>
+      <c r="F43" t="str">
+        <v>27th International Conference on Electrical Machines 2024 (ICEM 2026)</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Funchal, Portugal</v>
+      </c>
+      <c r="H43" t="str">
+        <v>2026.09</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B44" t="str">
+        <v>10</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2026</v>
+      </c>
+      <c r="D44" t="str">
+        <v>J. H. Lee, H. S. Kim, S. H. Park, J. C. Park, and M. S. Lim*</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Deep Transfer Learning-Assisted Fast Performance Prediction for AFPM considering PM Overhang Effects and Radial Leakage Flux</v>
+      </c>
+      <c r="F44" t="str">
+        <v>2026 International Conference on Magnetics (INTERMAG 2026)</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Manchester, United Kingdom</v>
+      </c>
+      <c r="H44" t="str">
+        <v>2026.04</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I44"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5510,7 +6582,7 @@
         <v>TRUE</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C2" t="str">
         <v>US</v>
@@ -5551,9 +6623,32 @@
         <v>US 11,757,383 B2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="B4" t="str">
+        <v>10</v>
+      </c>
+      <c r="C4" t="str">
+        <v>KOR</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Filed</v>
+      </c>
+      <c r="E4" t="str">
+        <v>매입형 영구자석 모터의 회전자(Rotor for Interior Permanent Magnet Motor)</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026</v>
+      </c>
+      <c r="G4" t="str">
+        <v>10-2026-0034283</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>